<commit_message>
Added Course Filter automation
</commit_message>
<xml_diff>
--- a/src/resources/data/CourseFilter.xlsx
+++ b/src/resources/data/CourseFilter.xlsx
@@ -12,7 +12,7 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="14380" windowHeight="4330" tabRatio="500"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Levels" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0" iterate="1" iterateCount="1000" iterateDelta="0.01"/>
 </workbook>
@@ -424,6 +424,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A5"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="15" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="12.54296875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">

</xml_diff>